<commit_message>
feat: make language rendering configuration-driven
</commit_message>
<xml_diff>
--- a/data/words.xlsx
+++ b/data/words.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Навчання\language-video-factory\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B604C510-C1D7-4D33-9F8B-08071BD62188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD0BFFF-9D84-4687-B7BB-2757BA48F567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12405" yWindow="90" windowWidth="16395" windowHeight="15510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>id</t>
   </si>
@@ -88,6 +88,15 @@
   </si>
   <si>
     <t>red apple isolated on white background</t>
+  </si>
+  <si>
+    <t>pl</t>
+  </si>
+  <si>
+    <t>Rower</t>
+  </si>
+  <si>
+    <t>Jabłko</t>
   </si>
 </sst>
 </file>
@@ -419,10 +428,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -442,13 +451,16 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -468,13 +480,16 @@
         <v>12</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -494,9 +509,12 @@
         <v>19</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Add Spanish language support
</commit_message>
<xml_diff>
--- a/data/words.xlsx
+++ b/data/words.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Навчання\language-video-factory\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD0BFFF-9D84-4687-B7BB-2757BA48F567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1308EDE1-CA8B-4198-92C3-A11DFFCF11D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="135" windowWidth="16395" windowHeight="15510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>id</t>
   </si>
@@ -97,6 +97,15 @@
   </si>
   <si>
     <t>Jabłko</t>
+  </si>
+  <si>
+    <t>es</t>
+  </si>
+  <si>
+    <t>Bicicleta</t>
+  </si>
+  <si>
+    <t>Manzana</t>
   </si>
 </sst>
 </file>
@@ -428,10 +437,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -454,13 +463,16 @@
         <v>21</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -483,13 +495,16 @@
         <v>22</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -512,9 +527,12 @@
         <v>23</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>